<commit_message>
Add bottom-up Cost Build-up (Bevmax quote) and Blended tabs
- Cost Build-up tab: bottom-up COGS from Bevmax co-pack quote OG2026-05-21 v15
  (40,500-can run, $1.21/can, $29.10/case); adders (allergen/freight) + 5/5%
  overhead -> COGS Direct & Indirect per case
- SKU P&L COGS rows now pull from the Cost Build-up outputs (no longer manual)
- Blended tab: volume-weighted P&L across all 11 channels, per SKU + total,
  with blended per-case economics
- Tab order: Dashboard, Blended, TTL, 3 SKUs, Cost Build-up
- Model re-verified end-to-end (cost ties to quote; COGS flows to P&L & Blended)

https://claude.ai/code/session_01LAQuYmgiTdaYENaC433uU1
</commit_message>
<xml_diff>
--- a/Organika_RTD_PL_Aug-Nov2026.xlsx
+++ b/Organika_RTD_PL_Aug-Nov2026.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TTL ORGANIKA RTD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lime Lemon" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Passion Fruit Pineapple" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Raspberry" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Blended" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TTL ORGANIKA RTD" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lime Lemon" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Passion Fruit Pineapple" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Raspberry" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cost Build-up" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +22,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0_);(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="\$#,##0_);&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00_);&quot;($&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +78,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
@@ -114,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -153,18 +162,15 @@
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,10 +178,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -185,6 +194,38 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1423,6 +1464,526 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ORGANIKA RTD — BLENDED (all channels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CDN $ | Volume-weighted average across all 11 channels | per case = 24 cans | Aug 1 – Nov 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>CDN $</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Lime Lemon</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Passion Fruit Pineapple</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Raspberry</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>PERIOD TOTALS (Aug 1 – Nov 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Physical Cases</t>
+        </is>
+      </c>
+      <c r="B7" s="5">
+        <f>'Lime Lemon'!M9</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>'Passion Fruit Pineapple'!M9</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>'Raspberry'!M9</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>'TTL ORGANIKA RTD'!M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B8" s="7">
+        <f>'Lime Lemon'!M10</f>
+        <v/>
+      </c>
+      <c r="C8" s="7">
+        <f>'Passion Fruit Pineapple'!M10</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>'Raspberry'!M10</f>
+        <v/>
+      </c>
+      <c r="E8" s="7">
+        <f>'TTL ORGANIKA RTD'!M10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Discounts</t>
+        </is>
+      </c>
+      <c r="B9" s="7">
+        <f>'Lime Lemon'!M11</f>
+        <v/>
+      </c>
+      <c r="C9" s="7">
+        <f>'Passion Fruit Pineapple'!M11</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>'Raspberry'!M11</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>'TTL ORGANIKA RTD'!M11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Net Sales</t>
+        </is>
+      </c>
+      <c r="B10" s="7">
+        <f>'Lime Lemon'!M12</f>
+        <v/>
+      </c>
+      <c r="C10" s="7">
+        <f>'Passion Fruit Pineapple'!M12</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>'Raspberry'!M12</f>
+        <v/>
+      </c>
+      <c r="E10" s="7">
+        <f>'TTL ORGANIKA RTD'!M12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    COGS Direct</t>
+        </is>
+      </c>
+      <c r="B11" s="7">
+        <f>'Lime Lemon'!M13</f>
+        <v/>
+      </c>
+      <c r="C11" s="7">
+        <f>'Passion Fruit Pineapple'!M13</f>
+        <v/>
+      </c>
+      <c r="D11" s="7">
+        <f>'Raspberry'!M13</f>
+        <v/>
+      </c>
+      <c r="E11" s="7">
+        <f>'TTL ORGANIKA RTD'!M13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    COGS Indirect</t>
+        </is>
+      </c>
+      <c r="B12" s="7">
+        <f>'Lime Lemon'!M14</f>
+        <v/>
+      </c>
+      <c r="C12" s="7">
+        <f>'Passion Fruit Pineapple'!M14</f>
+        <v/>
+      </c>
+      <c r="D12" s="7">
+        <f>'Raspberry'!M14</f>
+        <v/>
+      </c>
+      <c r="E12" s="7">
+        <f>'TTL ORGANIKA RTD'!M14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Cost of Sales</t>
+        </is>
+      </c>
+      <c r="B13" s="7">
+        <f>'Lime Lemon'!M15</f>
+        <v/>
+      </c>
+      <c r="C13" s="7">
+        <f>'Passion Fruit Pineapple'!M15</f>
+        <v/>
+      </c>
+      <c r="D13" s="7">
+        <f>'Raspberry'!M15</f>
+        <v/>
+      </c>
+      <c r="E13" s="7">
+        <f>'TTL ORGANIKA RTD'!M15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Gross Profit</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>'Lime Lemon'!M16</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
+        <f>'Passion Fruit Pineapple'!M16</f>
+        <v/>
+      </c>
+      <c r="D14" s="7">
+        <f>'Raspberry'!M16</f>
+        <v/>
+      </c>
+      <c r="E14" s="7">
+        <f>'TTL ORGANIKA RTD'!M16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>GP %</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>'Lime Lemon'!M17</f>
+        <v/>
+      </c>
+      <c r="C15" s="9">
+        <f>'Passion Fruit Pineapple'!M17</f>
+        <v/>
+      </c>
+      <c r="D15" s="9">
+        <f>'Raspberry'!M17</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>'TTL ORGANIKA RTD'!M17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>A&amp;P</t>
+        </is>
+      </c>
+      <c r="B16" s="7">
+        <f>'Lime Lemon'!M22</f>
+        <v/>
+      </c>
+      <c r="C16" s="7">
+        <f>'Passion Fruit Pineapple'!M22</f>
+        <v/>
+      </c>
+      <c r="D16" s="7">
+        <f>'Raspberry'!M22</f>
+        <v/>
+      </c>
+      <c r="E16" s="7">
+        <f>'TTL ORGANIKA RTD'!M22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Contrib After A&amp;P (CAAP)</t>
+        </is>
+      </c>
+      <c r="B17" s="7">
+        <f>'Lime Lemon'!M24</f>
+        <v/>
+      </c>
+      <c r="C17" s="7">
+        <f>'Passion Fruit Pineapple'!M24</f>
+        <v/>
+      </c>
+      <c r="D17" s="7">
+        <f>'Raspberry'!M24</f>
+        <v/>
+      </c>
+      <c r="E17" s="7">
+        <f>'TTL ORGANIKA RTD'!M24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>BLENDED PER CASE (avg across channels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Gross Rev / case</t>
+        </is>
+      </c>
+      <c r="B20" s="6">
+        <f>'Lime Lemon'!M26</f>
+        <v/>
+      </c>
+      <c r="C20" s="6">
+        <f>'Passion Fruit Pineapple'!M26</f>
+        <v/>
+      </c>
+      <c r="D20" s="6">
+        <f>'Raspberry'!M26</f>
+        <v/>
+      </c>
+      <c r="E20" s="6">
+        <f>'TTL ORGANIKA RTD'!M26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Discounts / case</t>
+        </is>
+      </c>
+      <c r="B21" s="6">
+        <f>'Lime Lemon'!M27</f>
+        <v/>
+      </c>
+      <c r="C21" s="6">
+        <f>'Passion Fruit Pineapple'!M27</f>
+        <v/>
+      </c>
+      <c r="D21" s="6">
+        <f>'Raspberry'!M27</f>
+        <v/>
+      </c>
+      <c r="E21" s="6">
+        <f>'TTL ORGANIKA RTD'!M27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Net Sales / case</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>'Lime Lemon'!M28</f>
+        <v/>
+      </c>
+      <c r="C22" s="6">
+        <f>'Passion Fruit Pineapple'!M28</f>
+        <v/>
+      </c>
+      <c r="D22" s="6">
+        <f>'Raspberry'!M28</f>
+        <v/>
+      </c>
+      <c r="E22" s="6">
+        <f>'TTL ORGANIKA RTD'!M28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>COGS / case</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>'Lime Lemon'!M31</f>
+        <v/>
+      </c>
+      <c r="C23" s="6">
+        <f>'Passion Fruit Pineapple'!M31</f>
+        <v/>
+      </c>
+      <c r="D23" s="6">
+        <f>'Raspberry'!M31</f>
+        <v/>
+      </c>
+      <c r="E23" s="6">
+        <f>'TTL ORGANIKA RTD'!M31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Gross Profit / case</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>'Lime Lemon'!M32</f>
+        <v/>
+      </c>
+      <c r="C24" s="6">
+        <f>'Passion Fruit Pineapple'!M32</f>
+        <v/>
+      </c>
+      <c r="D24" s="6">
+        <f>'Raspberry'!M32</f>
+        <v/>
+      </c>
+      <c r="E24" s="6">
+        <f>'TTL ORGANIKA RTD'!M32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>GP %</t>
+        </is>
+      </c>
+      <c r="B25" s="9">
+        <f>'Lime Lemon'!M33</f>
+        <v/>
+      </c>
+      <c r="C25" s="9">
+        <f>'Passion Fruit Pineapple'!M33</f>
+        <v/>
+      </c>
+      <c r="D25" s="9">
+        <f>'Raspberry'!M33</f>
+        <v/>
+      </c>
+      <c r="E25" s="9">
+        <f>'TTL ORGANIKA RTD'!M33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>A&amp;P / case</t>
+        </is>
+      </c>
+      <c r="B26" s="6">
+        <f>'Lime Lemon'!M34</f>
+        <v/>
+      </c>
+      <c r="C26" s="6">
+        <f>'Passion Fruit Pineapple'!M34</f>
+        <v/>
+      </c>
+      <c r="D26" s="6">
+        <f>'Raspberry'!M34</f>
+        <v/>
+      </c>
+      <c r="E26" s="6">
+        <f>'TTL ORGANIKA RTD'!M34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>CAAP / case</t>
+        </is>
+      </c>
+      <c r="B27" s="6">
+        <f>'Lime Lemon'!M35</f>
+        <v/>
+      </c>
+      <c r="C27" s="6">
+        <f>'Passion Fruit Pineapple'!M35</f>
+        <v/>
+      </c>
+      <c r="D27" s="6">
+        <f>'Raspberry'!M35</f>
+        <v/>
+      </c>
+      <c r="E27" s="6">
+        <f>'TTL ORGANIKA RTD'!M35</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A19:E19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF1F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1461,67 +2022,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="19" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="20" t="inlineStr">
+      <c r="M4" s="19" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1529,7 +2090,7 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
         </is>
@@ -1537,7 +2098,7 @@
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Organika RTD — All SKUs (Lime Lemon + Passion Fruit Pineapple + Raspberry)</t>
         </is>
@@ -2878,7 +3439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -2919,67 +3480,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="19" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="20" t="inlineStr">
+      <c r="M4" s="19" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2987,7 +3548,7 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
         </is>
@@ -2995,7 +3556,7 @@
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Organika RTD — Lime Lemon (6×4×355 ml)</t>
         </is>
@@ -3747,17 +4308,50 @@
           <t xml:space="preserve">    COGS Direct - per case</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="25" t="n"/>
-      <c r="G29" s="25" t="n"/>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
-      <c r="J29" s="25" t="n"/>
-      <c r="K29" s="25" t="n"/>
-      <c r="L29" s="25" t="n"/>
+      <c r="B29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="G29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="H29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="I29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
       <c r="M29" s="6">
         <f>IFERROR(M13/M9,"-")</f>
         <v/>
@@ -3769,17 +4363,50 @@
           <t xml:space="preserve">    COGS Indirect - per case</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="25" t="n"/>
-      <c r="G30" s="25" t="n"/>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
-      <c r="J30" s="25" t="n"/>
-      <c r="K30" s="25" t="n"/>
-      <c r="L30" s="25" t="n"/>
+      <c r="B30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="G30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="H30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="I30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
       <c r="M30" s="6">
         <f>IFERROR(M14/M9,"-")</f>
         <v/>
@@ -4072,7 +4699,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -4113,67 +4740,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="19" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="20" t="inlineStr">
+      <c r="M4" s="19" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4181,7 +4808,7 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
         </is>
@@ -4189,7 +4816,7 @@
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Organika RTD — Passion Fruit Pineapple (6×4×355 ml)</t>
         </is>
@@ -4941,17 +5568,50 @@
           <t xml:space="preserve">    COGS Direct - per case</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="25" t="n"/>
-      <c r="G29" s="25" t="n"/>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
-      <c r="J29" s="25" t="n"/>
-      <c r="K29" s="25" t="n"/>
-      <c r="L29" s="25" t="n"/>
+      <c r="B29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="G29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="H29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="I29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
       <c r="M29" s="6">
         <f>IFERROR(M13/M9,"-")</f>
         <v/>
@@ -4963,17 +5623,50 @@
           <t xml:space="preserve">    COGS Indirect - per case</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="25" t="n"/>
-      <c r="G30" s="25" t="n"/>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
-      <c r="J30" s="25" t="n"/>
-      <c r="K30" s="25" t="n"/>
-      <c r="L30" s="25" t="n"/>
+      <c r="B30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="G30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="H30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="I30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
       <c r="M30" s="6">
         <f>IFERROR(M14/M9,"-")</f>
         <v/>
@@ -5266,7 +5959,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFC00000"/>
@@ -5307,67 +6000,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="19" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="20" t="inlineStr">
+      <c r="M4" s="19" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -5375,7 +6068,7 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
         </is>
@@ -5383,7 +6076,7 @@
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Organika RTD — Raspberry (6×4×355 ml)</t>
         </is>
@@ -6135,17 +6828,50 @@
           <t xml:space="preserve">    COGS Direct - per case</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="25" t="n"/>
-      <c r="G29" s="25" t="n"/>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
-      <c r="J29" s="25" t="n"/>
-      <c r="K29" s="25" t="n"/>
-      <c r="L29" s="25" t="n"/>
+      <c r="B29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="G29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="H29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="I29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>'Cost Build-up'!$D$44</f>
+        <v/>
+      </c>
       <c r="M29" s="6">
         <f>IFERROR(M13/M9,"-")</f>
         <v/>
@@ -6157,17 +6883,50 @@
           <t xml:space="preserve">    COGS Indirect - per case</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="25" t="n"/>
-      <c r="G30" s="25" t="n"/>
-      <c r="H30" s="25" t="n"/>
-      <c r="I30" s="25" t="n"/>
-      <c r="J30" s="25" t="n"/>
-      <c r="K30" s="25" t="n"/>
-      <c r="L30" s="25" t="n"/>
+      <c r="B30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="G30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="H30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="I30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>'Cost Build-up'!$D$45</f>
+        <v/>
+      </c>
       <c r="M30" s="6">
         <f>IFERROR(M14/M9,"-")</f>
         <v/>
@@ -6458,4 +7217,612 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ORGANIKA RTD — BOTTOM-UP COST (Bevmax quote)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CDN $ | Quote OG2026-05-21 v15 (4-pk w/ sleeves) | Pack Summer 2026 | FOB Airdrie AB | excl. GST</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>RUN PARAMETERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Total run size</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>cans</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>40500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Number of SKUs</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>SKUs</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Cans per SKU</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>cans</t>
+        </is>
+      </c>
+      <c r="D8" s="5">
+        <f>D6/D7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Cans per case</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>cans</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Cans per 4-pack</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>cans</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Cases per run</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>cases</t>
+        </is>
+      </c>
+      <c r="D11" s="27">
+        <f>D6/D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>BEVMAX QUOTE — COST LINES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>Cost line</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>UofM</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Rate $</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>$/can</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tolling (blend/fill/pasteurize/carbonate)</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>per can</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>12150</v>
+      </c>
+      <c r="E15" s="6">
+        <f>D15/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    4-packing</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>per can</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E16" s="6">
+        <f>D16/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Skid packing</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>per run</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>439.45</v>
+      </c>
+      <c r="E17" s="6">
+        <f>D17/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Ingredients</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>per can</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>6480</v>
+      </c>
+      <c r="E18" s="6">
+        <f>D18/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Brite can + 202 LOE end</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>per can</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>12960</v>
+      </c>
+      <c r="E19" s="6">
+        <f>D19/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sleeves + application</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>per label</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <v>6601.5</v>
+      </c>
+      <c r="E20" s="6">
+        <f>D20/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sleeve-perforation setup (one-time)</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>per setup</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="n">
+        <v>489</v>
+      </c>
+      <c r="E21" s="6">
+        <f>D21/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    4-pk printed carton</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>per carton</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="n">
+        <v>0.411</v>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>6165</v>
+      </c>
+      <c r="E22" s="6">
+        <f>D22/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    24-pk white tray</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>per tray</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>1451.25</v>
+      </c>
+      <c r="E23" s="6">
+        <f>D23/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Grip sheets</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>per tray</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>175.78</v>
+      </c>
+      <c r="E24" s="6">
+        <f>D24/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tray labels</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>per tray</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>168.75</v>
+      </c>
+      <c r="E25" s="6">
+        <f>D25/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>Subtotal — Bevmax (FOB Airdrie)</t>
+        </is>
+      </c>
+      <c r="D26" s="33">
+        <f>SUM(D15:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="33">
+        <f>D26/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Bevmax cost / can</t>
+        </is>
+      </c>
+      <c r="D28" s="6">
+        <f>D26/$D$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Bevmax cost / 4-pack</t>
+        </is>
+      </c>
+      <c r="D29" s="6">
+        <f>D28*D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Bevmax cost / case (24)</t>
+        </is>
+      </c>
+      <c r="D30" s="33">
+        <f>D28*D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>ADDERS TO LANDED COST (per case)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Allergen handling (amortized)</t>
+        </is>
+      </c>
+      <c r="D33" s="6">
+        <f>167.5/D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Inbound freight to DC</t>
+        </is>
+      </c>
+      <c r="D34" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Testing / misc</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>OVERHEAD (% of landed direct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>OH cost %</t>
+        </is>
+      </c>
+      <c r="C38" s="34" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Other COGS %</t>
+        </is>
+      </c>
+      <c r="C39" s="34" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>→ COGS TO P&amp;L (per case)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="35" t="inlineStr">
+        <is>
+          <t>COGS Direct / case</t>
+        </is>
+      </c>
+      <c r="B44" s="36" t="n"/>
+      <c r="C44" s="36" t="n"/>
+      <c r="D44" s="37">
+        <f>D30+D33+D34+D35</f>
+        <v/>
+      </c>
+      <c r="E44" s="36" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>COGS Indirect / case</t>
+        </is>
+      </c>
+      <c r="B45" s="36" t="n"/>
+      <c r="C45" s="36" t="n"/>
+      <c r="D45" s="37">
+        <f>(C38+C39)*D44</f>
+        <v/>
+      </c>
+      <c r="E45" s="36" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>COGS Total / case</t>
+        </is>
+      </c>
+      <c r="B46" s="36" t="n"/>
+      <c r="C46" s="36" t="n"/>
+      <c r="D46" s="37">
+        <f>D44+D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="36" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>COGS / 4-pack</t>
+        </is>
+      </c>
+      <c r="D47" s="6">
+        <f>D46/D9*D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>COGS / can</t>
+        </is>
+      </c>
+      <c r="D48" s="6">
+        <f>D46/D9</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A13:E13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Scenarios/price-sensitivity tab and highlight all input cells
- New Scenarios tab: side-by-side CP (wholesale) x MSRP scenario comparison
  (Organika GP% + retailer margin%), a CP sensitivity ladder, and a CP x MSRP
  customer-margin heatmap grid; COGS pulled live from Cost Build-up
- Conditional-format heatmaps on margin rows/grids for quick read
- Every editable input cell now highlighted amber (FFFFF2CC) across all tabs;
  legend updated to 'yellow box = input'
- Verified: 16 scenario/sensitivity checks pass

https://claude.ai/code/session_01LAQuYmgiTdaYENaC433uU1
</commit_message>
<xml_diff>
--- a/Organika_RTD_PL_Aug-Nov2026.xlsx
+++ b/Organika_RTD_PL_Aug-Nov2026.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Blended" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TTL ORGANIKA RTD" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lime Lemon" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Passion Fruit Pineapple" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Raspberry" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cost Build-up" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Scenarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Blended" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TTL ORGANIKA RTD" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lime Lemon" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Passion Fruit Pineapple" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Raspberry" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cost Build-up" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="167" formatCode="\$#,##0.00_);&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +88,20 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +123,11 @@
         <fgColor rgb="FFEAF2FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -123,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -172,14 +190,39 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -187,13 +230,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -217,12 +254,6 @@
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1464,6 +1495,1230 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FFED7D31"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ORGANIKA RTD — SCENARIOS &amp; PRICE SENSITIVITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CDN $ per case (24 cans = 6 × 4-pack) | 🟡 yellow = edit | COGS pulled live from Cost Build-up ($D$46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SCENARIO COMPARISON  (CP = wholesale price, MSRP = shelf price)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Scenario 4</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Scenario 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CP — wholesale ($/case)</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>54</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>66</v>
+      </c>
+      <c r="E6" s="20" t="n"/>
+      <c r="F6" s="20" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>MSRP — retail ($/case)</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>84</v>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>96</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>108</v>
+      </c>
+      <c r="E7" s="20" t="n"/>
+      <c r="F7" s="20" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Promo / discount (% off CP)</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="21" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Volume (cases)</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>500</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>500</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>500</v>
+      </c>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>A&amp;P ($/case)</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="20" t="n"/>
+      <c r="F10" s="20" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Net price ($/case)</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>B6*(1-B8)</f>
+        <v/>
+      </c>
+      <c r="C11" s="6">
+        <f>C6*(1-C8)</f>
+        <v/>
+      </c>
+      <c r="D11" s="6">
+        <f>D6*(1-D8)</f>
+        <v/>
+      </c>
+      <c r="E11" s="6">
+        <f>E6*(1-E8)</f>
+        <v/>
+      </c>
+      <c r="F11" s="6">
+        <f>F6*(1-F8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>COGS ($/case)</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="D12" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Organika GP ($/case)</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <f>B11-B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="6">
+        <f>C11-C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="6">
+        <f>D11-D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="6">
+        <f>E11-E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>F11-F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Organika GP %</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>IFERROR(B13/B11,"-")</f>
+        <v/>
+      </c>
+      <c r="C14" s="9">
+        <f>IFERROR(C13/C11,"-")</f>
+        <v/>
+      </c>
+      <c r="D14" s="9">
+        <f>IFERROR(D13/D11,"-")</f>
+        <v/>
+      </c>
+      <c r="E14" s="9">
+        <f>IFERROR(E13/E11,"-")</f>
+        <v/>
+      </c>
+      <c r="F14" s="9">
+        <f>IFERROR(F13/F11,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Customer margin %</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>IFERROR((B7-B6)/B7,"-")</f>
+        <v/>
+      </c>
+      <c r="C15" s="9">
+        <f>IFERROR((C7-C6)/C7,"-")</f>
+        <v/>
+      </c>
+      <c r="D15" s="9">
+        <f>IFERROR((D7-D6)/D7,"-")</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>IFERROR((E7-E6)/E7,"-")</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>IFERROR((F7-F6)/F7,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CAAP ($/case)</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>B13-B10</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>C13-C10</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>D13-D10</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>E13-E10</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>F13-F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>— per-pack &amp; period —</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>CP / 4-pack</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>B6/6</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>C6/6</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>D6/6</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>E6/6</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>F6/6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MSRP / 4-pack</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>B7/6</f>
+        <v/>
+      </c>
+      <c r="C19" s="6">
+        <f>C7/6</f>
+        <v/>
+      </c>
+      <c r="D19" s="6">
+        <f>D7/6</f>
+        <v/>
+      </c>
+      <c r="E19" s="6">
+        <f>E7/6</f>
+        <v/>
+      </c>
+      <c r="F19" s="6">
+        <f>F7/6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Net sales — period ($)</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>B11*B9</f>
+        <v/>
+      </c>
+      <c r="C20" s="7">
+        <f>C11*C9</f>
+        <v/>
+      </c>
+      <c r="D20" s="7">
+        <f>D11*D9</f>
+        <v/>
+      </c>
+      <c r="E20" s="7">
+        <f>E11*E9</f>
+        <v/>
+      </c>
+      <c r="F20" s="7">
+        <f>F11*F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Gross profit — period ($)</t>
+        </is>
+      </c>
+      <c r="B21" s="7">
+        <f>B13*B9</f>
+        <v/>
+      </c>
+      <c r="C21" s="7">
+        <f>C13*C9</f>
+        <v/>
+      </c>
+      <c r="D21" s="7">
+        <f>D13*D9</f>
+        <v/>
+      </c>
+      <c r="E21" s="7">
+        <f>E13*E9</f>
+        <v/>
+      </c>
+      <c r="F21" s="7">
+        <f>F13*F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>CAAP — period ($)</t>
+        </is>
+      </c>
+      <c r="B22" s="7">
+        <f>B16*B9</f>
+        <v/>
+      </c>
+      <c r="C22" s="7">
+        <f>C16*C9</f>
+        <v/>
+      </c>
+      <c r="D22" s="7">
+        <f>D16*D9</f>
+        <v/>
+      </c>
+      <c r="E22" s="7">
+        <f>E16*E9</f>
+        <v/>
+      </c>
+      <c r="F22" s="7">
+        <f>F16*F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>PRICE SENSITIVITY — Organika margin as CP varies</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>CP start ($/case)</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>step ($)</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="25" t="inlineStr">
+        <is>
+          <t>ref MSRP ($/case)</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>96</v>
+      </c>
+      <c r="G25" s="25" t="inlineStr">
+        <is>
+          <t>promo %</t>
+        </is>
+      </c>
+      <c r="H25" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>CP /case</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>CP /4-pack</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Net /case</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>COGS /case</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>GP /case</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>GP %</t>
+        </is>
+      </c>
+      <c r="G26" s="26" t="inlineStr">
+        <is>
+          <t>Cust margin %</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6">
+        <f>$B$25+0*$D$25</f>
+        <v/>
+      </c>
+      <c r="B27" s="6">
+        <f>A27/6</f>
+        <v/>
+      </c>
+      <c r="C27" s="6">
+        <f>A27*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D27" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E27" s="6">
+        <f>C27-D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="13">
+        <f>IFERROR(E27/C27,"-")</f>
+        <v/>
+      </c>
+      <c r="G27" s="13">
+        <f>IFERROR(($F$25-A27)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6">
+        <f>$B$25+1*$D$25</f>
+        <v/>
+      </c>
+      <c r="B28" s="6">
+        <f>A28/6</f>
+        <v/>
+      </c>
+      <c r="C28" s="6">
+        <f>A28*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D28" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E28" s="6">
+        <f>C28-D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="13">
+        <f>IFERROR(E28/C28,"-")</f>
+        <v/>
+      </c>
+      <c r="G28" s="13">
+        <f>IFERROR(($F$25-A28)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6">
+        <f>$B$25+2*$D$25</f>
+        <v/>
+      </c>
+      <c r="B29" s="6">
+        <f>A29/6</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>A29*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>C29-D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="13">
+        <f>IFERROR(E29/C29,"-")</f>
+        <v/>
+      </c>
+      <c r="G29" s="13">
+        <f>IFERROR(($F$25-A29)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6">
+        <f>$B$25+3*$D$25</f>
+        <v/>
+      </c>
+      <c r="B30" s="6">
+        <f>A30/6</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>A30*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>C30-D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="13">
+        <f>IFERROR(E30/C30,"-")</f>
+        <v/>
+      </c>
+      <c r="G30" s="13">
+        <f>IFERROR(($F$25-A30)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6">
+        <f>$B$25+4*$D$25</f>
+        <v/>
+      </c>
+      <c r="B31" s="6">
+        <f>A31/6</f>
+        <v/>
+      </c>
+      <c r="C31" s="6">
+        <f>A31*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D31" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E31" s="6">
+        <f>C31-D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="13">
+        <f>IFERROR(E31/C31,"-")</f>
+        <v/>
+      </c>
+      <c r="G31" s="13">
+        <f>IFERROR(($F$25-A31)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6">
+        <f>$B$25+5*$D$25</f>
+        <v/>
+      </c>
+      <c r="B32" s="6">
+        <f>A32/6</f>
+        <v/>
+      </c>
+      <c r="C32" s="6">
+        <f>A32*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D32" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E32" s="6">
+        <f>C32-D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="13">
+        <f>IFERROR(E32/C32,"-")</f>
+        <v/>
+      </c>
+      <c r="G32" s="13">
+        <f>IFERROR(($F$25-A32)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6">
+        <f>$B$25+6*$D$25</f>
+        <v/>
+      </c>
+      <c r="B33" s="6">
+        <f>A33/6</f>
+        <v/>
+      </c>
+      <c r="C33" s="6">
+        <f>A33*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D33" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E33" s="6">
+        <f>C33-D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="13">
+        <f>IFERROR(E33/C33,"-")</f>
+        <v/>
+      </c>
+      <c r="G33" s="13">
+        <f>IFERROR(($F$25-A33)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6">
+        <f>$B$25+7*$D$25</f>
+        <v/>
+      </c>
+      <c r="B34" s="6">
+        <f>A34/6</f>
+        <v/>
+      </c>
+      <c r="C34" s="6">
+        <f>A34*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D34" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E34" s="6">
+        <f>C34-D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="13">
+        <f>IFERROR(E34/C34,"-")</f>
+        <v/>
+      </c>
+      <c r="G34" s="13">
+        <f>IFERROR(($F$25-A34)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6">
+        <f>$B$25+8*$D$25</f>
+        <v/>
+      </c>
+      <c r="B35" s="6">
+        <f>A35/6</f>
+        <v/>
+      </c>
+      <c r="C35" s="6">
+        <f>A35*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D35" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E35" s="6">
+        <f>C35-D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="13">
+        <f>IFERROR(E35/C35,"-")</f>
+        <v/>
+      </c>
+      <c r="G35" s="13">
+        <f>IFERROR(($F$25-A35)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6">
+        <f>$B$25+9*$D$25</f>
+        <v/>
+      </c>
+      <c r="B36" s="6">
+        <f>A36/6</f>
+        <v/>
+      </c>
+      <c r="C36" s="6">
+        <f>A36*(1-$H$25)</f>
+        <v/>
+      </c>
+      <c r="D36" s="6">
+        <f>'Cost Build-up'!$D$46</f>
+        <v/>
+      </c>
+      <c r="E36" s="6">
+        <f>C36-D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="13">
+        <f>IFERROR(E36/C36,"-")</f>
+        <v/>
+      </c>
+      <c r="G36" s="13">
+        <f>IFERROR(($F$25-A36)/$F$25,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>CUSTOMER (RETAILER) MARGIN %  —  CP (down) × MSRP (across)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>CP ↓  /  MSRP →</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
+        <v>84</v>
+      </c>
+      <c r="C40" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="D40" s="20" t="n">
+        <v>96</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>102</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <v>108</v>
+      </c>
+      <c r="G40" s="20" t="n">
+        <v>114</v>
+      </c>
+      <c r="H40" s="20" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6">
+        <f>$B$25+0*$D$25</f>
+        <v/>
+      </c>
+      <c r="B41" s="13">
+        <f>IFERROR((B$40-$A41)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C41" s="13">
+        <f>IFERROR((C$40-$A41)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D41" s="13">
+        <f>IFERROR((D$40-$A41)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E41" s="13">
+        <f>IFERROR((E$40-$A41)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F41" s="13">
+        <f>IFERROR((F$40-$A41)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G41" s="13">
+        <f>IFERROR((G$40-$A41)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H41" s="13">
+        <f>IFERROR((H$40-$A41)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6">
+        <f>$B$25+1*$D$25</f>
+        <v/>
+      </c>
+      <c r="B42" s="13">
+        <f>IFERROR((B$40-$A42)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C42" s="13">
+        <f>IFERROR((C$40-$A42)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D42" s="13">
+        <f>IFERROR((D$40-$A42)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E42" s="13">
+        <f>IFERROR((E$40-$A42)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F42" s="13">
+        <f>IFERROR((F$40-$A42)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G42" s="13">
+        <f>IFERROR((G$40-$A42)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H42" s="13">
+        <f>IFERROR((H$40-$A42)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6">
+        <f>$B$25+2*$D$25</f>
+        <v/>
+      </c>
+      <c r="B43" s="13">
+        <f>IFERROR((B$40-$A43)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C43" s="13">
+        <f>IFERROR((C$40-$A43)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D43" s="13">
+        <f>IFERROR((D$40-$A43)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E43" s="13">
+        <f>IFERROR((E$40-$A43)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F43" s="13">
+        <f>IFERROR((F$40-$A43)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G43" s="13">
+        <f>IFERROR((G$40-$A43)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H43" s="13">
+        <f>IFERROR((H$40-$A43)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6">
+        <f>$B$25+3*$D$25</f>
+        <v/>
+      </c>
+      <c r="B44" s="13">
+        <f>IFERROR((B$40-$A44)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C44" s="13">
+        <f>IFERROR((C$40-$A44)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D44" s="13">
+        <f>IFERROR((D$40-$A44)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E44" s="13">
+        <f>IFERROR((E$40-$A44)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F44" s="13">
+        <f>IFERROR((F$40-$A44)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G44" s="13">
+        <f>IFERROR((G$40-$A44)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H44" s="13">
+        <f>IFERROR((H$40-$A44)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6">
+        <f>$B$25+4*$D$25</f>
+        <v/>
+      </c>
+      <c r="B45" s="13">
+        <f>IFERROR((B$40-$A45)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C45" s="13">
+        <f>IFERROR((C$40-$A45)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D45" s="13">
+        <f>IFERROR((D$40-$A45)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E45" s="13">
+        <f>IFERROR((E$40-$A45)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F45" s="13">
+        <f>IFERROR((F$40-$A45)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G45" s="13">
+        <f>IFERROR((G$40-$A45)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H45" s="13">
+        <f>IFERROR((H$40-$A45)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6">
+        <f>$B$25+5*$D$25</f>
+        <v/>
+      </c>
+      <c r="B46" s="13">
+        <f>IFERROR((B$40-$A46)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C46" s="13">
+        <f>IFERROR((C$40-$A46)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D46" s="13">
+        <f>IFERROR((D$40-$A46)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E46" s="13">
+        <f>IFERROR((E$40-$A46)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F46" s="13">
+        <f>IFERROR((F$40-$A46)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G46" s="13">
+        <f>IFERROR((G$40-$A46)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H46" s="13">
+        <f>IFERROR((H$40-$A46)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6">
+        <f>$B$25+6*$D$25</f>
+        <v/>
+      </c>
+      <c r="B47" s="13">
+        <f>IFERROR((B$40-$A47)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C47" s="13">
+        <f>IFERROR((C$40-$A47)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D47" s="13">
+        <f>IFERROR((D$40-$A47)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E47" s="13">
+        <f>IFERROR((E$40-$A47)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F47" s="13">
+        <f>IFERROR((F$40-$A47)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G47" s="13">
+        <f>IFERROR((G$40-$A47)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H47" s="13">
+        <f>IFERROR((H$40-$A47)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6">
+        <f>$B$25+7*$D$25</f>
+        <v/>
+      </c>
+      <c r="B48" s="13">
+        <f>IFERROR((B$40-$A48)/B$40,"-")</f>
+        <v/>
+      </c>
+      <c r="C48" s="13">
+        <f>IFERROR((C$40-$A48)/C$40,"-")</f>
+        <v/>
+      </c>
+      <c r="D48" s="13">
+        <f>IFERROR((D$40-$A48)/D$40,"-")</f>
+        <v/>
+      </c>
+      <c r="E48" s="13">
+        <f>IFERROR((E$40-$A48)/E$40,"-")</f>
+        <v/>
+      </c>
+      <c r="F48" s="13">
+        <f>IFERROR((F$40-$A48)/F$40,"-")</f>
+        <v/>
+      </c>
+      <c r="G48" s="13">
+        <f>IFERROR((G$40-$A48)/G$40,"-")</f>
+        <v/>
+      </c>
+      <c r="H48" s="13">
+        <f>IFERROR((H$40-$A48)/H$40,"-")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B14:F14">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.35"/>
+        <cfvo type="num" val="0.7"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:F15">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.35"/>
+        <cfvo type="num" val="0.7"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F27:F36">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.35"/>
+        <cfvo type="num" val="0.7"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27:G36">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.35"/>
+        <cfvo type="num" val="0.7"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B41:H48">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.3"/>
+        <cfvo type="num" val="0.5"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF7030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1498,29 +2753,29 @@
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Lime Lemon</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Passion Fruit Pineapple</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>Raspberry</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>PERIOD TOTALS (Aug 1 – Nov 1)</t>
         </is>
@@ -1780,7 +3035,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>BLENDED PER CASE (avg across channels)</t>
         </is>
@@ -1981,7 +3236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF1F3864"/>
@@ -2022,67 +3277,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="28" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="I4" s="28" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="J4" s="28" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="28" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="18" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="19" t="inlineStr">
+      <c r="M4" s="29" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2090,15 +3345,15 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Yellow box = input (edit these)   ⚫ Black = formula   🔵 Blue band = margin %</t>
         </is>
       </c>
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Organika RTD — All SKUs (Lime Lemon + Passion Fruit Pineapple + Raspberry)</t>
         </is>
@@ -3439,7 +4694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -3480,67 +4735,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="28" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="I4" s="28" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="J4" s="28" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="28" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="18" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="19" t="inlineStr">
+      <c r="M4" s="29" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -3548,15 +4803,15 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Yellow box = input (edit these)   ⚫ Black = formula   🔵 Blue band = margin %</t>
         </is>
       </c>
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Organika RTD — Lime Lemon (6×4×355 ml)</t>
         </is>
@@ -3568,17 +4823,17 @@
           <t>Physical Cases</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="23" t="n"/>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="23" t="n"/>
-      <c r="G9" s="23" t="n"/>
-      <c r="H9" s="23" t="n"/>
-      <c r="I9" s="23" t="n"/>
-      <c r="J9" s="23" t="n"/>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="23" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="22" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="22" t="n"/>
+      <c r="L9" s="22" t="n"/>
       <c r="M9" s="5">
         <f>SUM(B9:L9)</f>
         <v/>
@@ -4031,17 +5286,17 @@
           <t xml:space="preserve">    A&amp;P Consumer</t>
         </is>
       </c>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="24" t="n"/>
-      <c r="K19" s="24" t="n"/>
-      <c r="L19" s="24" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+      <c r="J19" s="32" t="n"/>
+      <c r="K19" s="32" t="n"/>
+      <c r="L19" s="32" t="n"/>
       <c r="M19" s="7">
         <f>SUM(B19:L19)</f>
         <v/>
@@ -4053,17 +5308,17 @@
           <t xml:space="preserve">    A&amp;P Trade</t>
         </is>
       </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
-      <c r="L20" s="24" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="32" t="n"/>
+      <c r="K20" s="32" t="n"/>
+      <c r="L20" s="32" t="n"/>
       <c r="M20" s="7">
         <f>SUM(B20:L20)</f>
         <v/>
@@ -4075,17 +5330,17 @@
           <t xml:space="preserve">    A&amp;P Sales</t>
         </is>
       </c>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="24" t="n"/>
-      <c r="K21" s="24" t="n"/>
-      <c r="L21" s="24" t="n"/>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n"/>
+      <c r="K21" s="32" t="n"/>
+      <c r="L21" s="32" t="n"/>
       <c r="M21" s="7">
         <f>SUM(B21:L21)</f>
         <v/>
@@ -4209,17 +5464,17 @@
           <t>Gross Rev - per case</t>
         </is>
       </c>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="25" t="n"/>
-      <c r="D26" s="25" t="n"/>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="25" t="n"/>
-      <c r="G26" s="25" t="n"/>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="25" t="n"/>
-      <c r="K26" s="25" t="n"/>
-      <c r="L26" s="25" t="n"/>
+      <c r="B26" s="20" t="n"/>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="20" t="n"/>
+      <c r="F26" s="20" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="20" t="n"/>
+      <c r="J26" s="20" t="n"/>
+      <c r="K26" s="20" t="n"/>
+      <c r="L26" s="20" t="n"/>
       <c r="M26" s="6">
         <f>IFERROR(M10/M9,"-")</f>
         <v/>
@@ -4231,17 +5486,17 @@
           <t>Discounts - per case</t>
         </is>
       </c>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="25" t="n"/>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="25" t="n"/>
-      <c r="G27" s="25" t="n"/>
-      <c r="H27" s="25" t="n"/>
-      <c r="I27" s="25" t="n"/>
-      <c r="J27" s="25" t="n"/>
-      <c r="K27" s="25" t="n"/>
-      <c r="L27" s="25" t="n"/>
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
+      <c r="J27" s="20" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="20" t="n"/>
       <c r="M27" s="6">
         <f>IFERROR(M11/M9,"-")</f>
         <v/>
@@ -4699,7 +5954,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -4740,67 +5995,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="28" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="I4" s="28" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="J4" s="28" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="28" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="18" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="19" t="inlineStr">
+      <c r="M4" s="29" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4808,15 +6063,15 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Yellow box = input (edit these)   ⚫ Black = formula   🔵 Blue band = margin %</t>
         </is>
       </c>
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Organika RTD — Passion Fruit Pineapple (6×4×355 ml)</t>
         </is>
@@ -4828,17 +6083,17 @@
           <t>Physical Cases</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="23" t="n"/>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="23" t="n"/>
-      <c r="G9" s="23" t="n"/>
-      <c r="H9" s="23" t="n"/>
-      <c r="I9" s="23" t="n"/>
-      <c r="J9" s="23" t="n"/>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="23" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="22" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="22" t="n"/>
+      <c r="L9" s="22" t="n"/>
       <c r="M9" s="5">
         <f>SUM(B9:L9)</f>
         <v/>
@@ -5291,17 +6546,17 @@
           <t xml:space="preserve">    A&amp;P Consumer</t>
         </is>
       </c>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="24" t="n"/>
-      <c r="K19" s="24" t="n"/>
-      <c r="L19" s="24" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+      <c r="J19" s="32" t="n"/>
+      <c r="K19" s="32" t="n"/>
+      <c r="L19" s="32" t="n"/>
       <c r="M19" s="7">
         <f>SUM(B19:L19)</f>
         <v/>
@@ -5313,17 +6568,17 @@
           <t xml:space="preserve">    A&amp;P Trade</t>
         </is>
       </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
-      <c r="L20" s="24" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="32" t="n"/>
+      <c r="K20" s="32" t="n"/>
+      <c r="L20" s="32" t="n"/>
       <c r="M20" s="7">
         <f>SUM(B20:L20)</f>
         <v/>
@@ -5335,17 +6590,17 @@
           <t xml:space="preserve">    A&amp;P Sales</t>
         </is>
       </c>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="24" t="n"/>
-      <c r="K21" s="24" t="n"/>
-      <c r="L21" s="24" t="n"/>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n"/>
+      <c r="K21" s="32" t="n"/>
+      <c r="L21" s="32" t="n"/>
       <c r="M21" s="7">
         <f>SUM(B21:L21)</f>
         <v/>
@@ -5469,17 +6724,17 @@
           <t>Gross Rev - per case</t>
         </is>
       </c>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="25" t="n"/>
-      <c r="D26" s="25" t="n"/>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="25" t="n"/>
-      <c r="G26" s="25" t="n"/>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="25" t="n"/>
-      <c r="K26" s="25" t="n"/>
-      <c r="L26" s="25" t="n"/>
+      <c r="B26" s="20" t="n"/>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="20" t="n"/>
+      <c r="F26" s="20" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="20" t="n"/>
+      <c r="J26" s="20" t="n"/>
+      <c r="K26" s="20" t="n"/>
+      <c r="L26" s="20" t="n"/>
       <c r="M26" s="6">
         <f>IFERROR(M10/M9,"-")</f>
         <v/>
@@ -5491,17 +6746,17 @@
           <t>Discounts - per case</t>
         </is>
       </c>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="25" t="n"/>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="25" t="n"/>
-      <c r="G27" s="25" t="n"/>
-      <c r="H27" s="25" t="n"/>
-      <c r="I27" s="25" t="n"/>
-      <c r="J27" s="25" t="n"/>
-      <c r="K27" s="25" t="n"/>
-      <c r="L27" s="25" t="n"/>
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
+      <c r="J27" s="20" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="20" t="n"/>
       <c r="M27" s="6">
         <f>IFERROR(M11/M9,"-")</f>
         <v/>
@@ -5959,7 +7214,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFC00000"/>
@@ -6000,67 +7255,67 @@
     </row>
     <row r="3" ht="7.5" customHeight="1"/>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>CDN $</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>On-premise</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>Corporate Office</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="28" t="inlineStr">
         <is>
           <t>Purity Life</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="I4" s="28" t="inlineStr">
         <is>
           <t>Natural &amp; Specialty Direct</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="J4" s="28" t="inlineStr">
         <is>
           <t>FDM Direct</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="28" t="inlineStr">
         <is>
           <t>Convenience</t>
         </is>
       </c>
-      <c r="L4" s="18" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr">
         <is>
           <t>Fitness Centre</t>
         </is>
       </c>
-      <c r="M4" s="19" t="inlineStr">
+      <c r="M4" s="29" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -6068,15 +7323,15 @@
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="13.5" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>🔵 Blue = input cell (hardcoded)   ⚫ Black = formula   🔵 Light-blue band = margin %</t>
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>🟡 Yellow box = input (edit these)   ⚫ Black = formula   🔵 Blue band = margin %</t>
         </is>
       </c>
     </row>
     <row r="7" ht="7.5" customHeight="1"/>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Organika RTD — Raspberry (6×4×355 ml)</t>
         </is>
@@ -6088,17 +7343,17 @@
           <t>Physical Cases</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="23" t="n"/>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="23" t="n"/>
-      <c r="G9" s="23" t="n"/>
-      <c r="H9" s="23" t="n"/>
-      <c r="I9" s="23" t="n"/>
-      <c r="J9" s="23" t="n"/>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="23" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="22" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="22" t="n"/>
+      <c r="L9" s="22" t="n"/>
       <c r="M9" s="5">
         <f>SUM(B9:L9)</f>
         <v/>
@@ -6551,17 +7806,17 @@
           <t xml:space="preserve">    A&amp;P Consumer</t>
         </is>
       </c>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="24" t="n"/>
-      <c r="K19" s="24" t="n"/>
-      <c r="L19" s="24" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+      <c r="J19" s="32" t="n"/>
+      <c r="K19" s="32" t="n"/>
+      <c r="L19" s="32" t="n"/>
       <c r="M19" s="7">
         <f>SUM(B19:L19)</f>
         <v/>
@@ -6573,17 +7828,17 @@
           <t xml:space="preserve">    A&amp;P Trade</t>
         </is>
       </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
-      <c r="L20" s="24" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="32" t="n"/>
+      <c r="K20" s="32" t="n"/>
+      <c r="L20" s="32" t="n"/>
       <c r="M20" s="7">
         <f>SUM(B20:L20)</f>
         <v/>
@@ -6595,17 +7850,17 @@
           <t xml:space="preserve">    A&amp;P Sales</t>
         </is>
       </c>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="24" t="n"/>
-      <c r="K21" s="24" t="n"/>
-      <c r="L21" s="24" t="n"/>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n"/>
+      <c r="K21" s="32" t="n"/>
+      <c r="L21" s="32" t="n"/>
       <c r="M21" s="7">
         <f>SUM(B21:L21)</f>
         <v/>
@@ -6729,17 +7984,17 @@
           <t>Gross Rev - per case</t>
         </is>
       </c>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="25" t="n"/>
-      <c r="D26" s="25" t="n"/>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="25" t="n"/>
-      <c r="G26" s="25" t="n"/>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="25" t="n"/>
-      <c r="K26" s="25" t="n"/>
-      <c r="L26" s="25" t="n"/>
+      <c r="B26" s="20" t="n"/>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="20" t="n"/>
+      <c r="F26" s="20" t="n"/>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="20" t="n"/>
+      <c r="J26" s="20" t="n"/>
+      <c r="K26" s="20" t="n"/>
+      <c r="L26" s="20" t="n"/>
       <c r="M26" s="6">
         <f>IFERROR(M10/M9,"-")</f>
         <v/>
@@ -6751,17 +8006,17 @@
           <t>Discounts - per case</t>
         </is>
       </c>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="25" t="n"/>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="25" t="n"/>
-      <c r="G27" s="25" t="n"/>
-      <c r="H27" s="25" t="n"/>
-      <c r="I27" s="25" t="n"/>
-      <c r="J27" s="25" t="n"/>
-      <c r="K27" s="25" t="n"/>
-      <c r="L27" s="25" t="n"/>
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
+      <c r="J27" s="20" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="20" t="n"/>
       <c r="M27" s="6">
         <f>IFERROR(M11/M9,"-")</f>
         <v/>
@@ -7219,7 +8474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF548235"/>
@@ -7263,12 +8518,12 @@
           <t>Total run size</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>cans</t>
         </is>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="22" t="n">
         <v>40500</v>
       </c>
     </row>
@@ -7278,12 +8533,12 @@
           <t>Number of SKUs</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>SKUs</t>
         </is>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7293,7 +8548,7 @@
           <t>Cans per SKU</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>cans</t>
         </is>
@@ -7309,12 +8564,12 @@
           <t>Cans per case</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="33" t="inlineStr">
         <is>
           <t>cans</t>
         </is>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="22" t="n">
         <v>24</v>
       </c>
     </row>
@@ -7324,12 +8579,12 @@
           <t>Cans per 4-pack</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>cans</t>
         </is>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="22" t="n">
         <v>4</v>
       </c>
     </row>
@@ -7339,12 +8594,12 @@
           <t>Cases per run</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="33" t="inlineStr">
         <is>
           <t>cases</t>
         </is>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="34">
         <f>D6/D9</f>
         <v/>
       </c>
@@ -7357,27 +8612,27 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>Cost line</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="36" t="inlineStr">
         <is>
           <t>UofM</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="36" t="inlineStr">
         <is>
           <t>Rate $</t>
         </is>
       </c>
-      <c r="D14" s="29" t="inlineStr">
+      <c r="D14" s="36" t="inlineStr">
         <is>
           <t>Total $</t>
         </is>
       </c>
-      <c r="E14" s="29" t="inlineStr">
+      <c r="E14" s="36" t="inlineStr">
         <is>
           <t>$/can</t>
         </is>
@@ -7389,15 +8644,15 @@
           <t xml:space="preserve">    Tolling (blend/fill/pasteurize/carbonate)</t>
         </is>
       </c>
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="37" t="inlineStr">
         <is>
           <t>per can</t>
         </is>
       </c>
-      <c r="C15" s="25" t="n">
+      <c r="C15" s="20" t="n">
         <v>0.3</v>
       </c>
-      <c r="D15" s="25" t="n">
+      <c r="D15" s="20" t="n">
         <v>12150</v>
       </c>
       <c r="E15" s="6">
@@ -7411,15 +8666,15 @@
           <t xml:space="preserve">    4-packing</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="37" t="inlineStr">
         <is>
           <t>per can</t>
         </is>
       </c>
-      <c r="C16" s="25" t="n">
+      <c r="C16" s="20" t="n">
         <v>0.05</v>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D16" s="20" t="n">
         <v>2025</v>
       </c>
       <c r="E16" s="6">
@@ -7433,17 +8688,17 @@
           <t xml:space="preserve">    Skid packing</t>
         </is>
       </c>
-      <c r="B17" s="30" t="inlineStr">
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>per run</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="20" t="n">
         <v>439.45</v>
       </c>
       <c r="E17" s="6">
@@ -7457,15 +8712,15 @@
           <t xml:space="preserve">    Ingredients</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="37" t="inlineStr">
         <is>
           <t>per can</t>
         </is>
       </c>
-      <c r="C18" s="25" t="n">
+      <c r="C18" s="20" t="n">
         <v>0.16</v>
       </c>
-      <c r="D18" s="25" t="n">
+      <c r="D18" s="20" t="n">
         <v>6480</v>
       </c>
       <c r="E18" s="6">
@@ -7479,15 +8734,15 @@
           <t xml:space="preserve">    Brite can + 202 LOE end</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr">
+      <c r="B19" s="37" t="inlineStr">
         <is>
           <t>per can</t>
         </is>
       </c>
-      <c r="C19" s="25" t="n">
+      <c r="C19" s="20" t="n">
         <v>0.32</v>
       </c>
-      <c r="D19" s="25" t="n">
+      <c r="D19" s="20" t="n">
         <v>12960</v>
       </c>
       <c r="E19" s="6">
@@ -7501,15 +8756,15 @@
           <t xml:space="preserve">    Sleeves + application</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="37" t="inlineStr">
         <is>
           <t>per label</t>
         </is>
       </c>
-      <c r="C20" s="25" t="n">
+      <c r="C20" s="20" t="n">
         <v>0.163</v>
       </c>
-      <c r="D20" s="25" t="n">
+      <c r="D20" s="20" t="n">
         <v>6601.5</v>
       </c>
       <c r="E20" s="6">
@@ -7523,17 +8778,17 @@
           <t xml:space="preserve">    Sleeve-perforation setup (one-time)</t>
         </is>
       </c>
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>per setup</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D21" s="25" t="n">
+      <c r="D21" s="20" t="n">
         <v>489</v>
       </c>
       <c r="E21" s="6">
@@ -7547,15 +8802,15 @@
           <t xml:space="preserve">    4-pk printed carton</t>
         </is>
       </c>
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="37" t="inlineStr">
         <is>
           <t>per carton</t>
         </is>
       </c>
-      <c r="C22" s="25" t="n">
+      <c r="C22" s="20" t="n">
         <v>0.411</v>
       </c>
-      <c r="D22" s="25" t="n">
+      <c r="D22" s="20" t="n">
         <v>6165</v>
       </c>
       <c r="E22" s="6">
@@ -7569,15 +8824,15 @@
           <t xml:space="preserve">    24-pk white tray</t>
         </is>
       </c>
-      <c r="B23" s="30" t="inlineStr">
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>per tray</t>
         </is>
       </c>
-      <c r="C23" s="25" t="n">
+      <c r="C23" s="20" t="n">
         <v>0.86</v>
       </c>
-      <c r="D23" s="25" t="n">
+      <c r="D23" s="20" t="n">
         <v>1451.25</v>
       </c>
       <c r="E23" s="6">
@@ -7591,15 +8846,15 @@
           <t xml:space="preserve">    Grip sheets</t>
         </is>
       </c>
-      <c r="B24" s="30" t="inlineStr">
+      <c r="B24" s="37" t="inlineStr">
         <is>
           <t>per tray</t>
         </is>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="C24" s="20" t="n">
         <v>1.25</v>
       </c>
-      <c r="D24" s="25" t="n">
+      <c r="D24" s="20" t="n">
         <v>175.78</v>
       </c>
       <c r="E24" s="6">
@@ -7613,15 +8868,15 @@
           <t xml:space="preserve">    Tray labels</t>
         </is>
       </c>
-      <c r="B25" s="30" t="inlineStr">
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>per tray</t>
         </is>
       </c>
-      <c r="C25" s="25" t="n">
+      <c r="C25" s="20" t="n">
         <v>0.05</v>
       </c>
-      <c r="D25" s="25" t="n">
+      <c r="D25" s="20" t="n">
         <v>168.75</v>
       </c>
       <c r="E25" s="6">
@@ -7630,16 +8885,16 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" s="39" t="inlineStr">
         <is>
           <t>Subtotal — Bevmax (FOB Airdrie)</t>
         </is>
       </c>
-      <c r="D26" s="33">
+      <c r="D26" s="40">
         <f>SUM(D15:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="33">
+      <c r="E26" s="40">
         <f>D26/$D$6</f>
         <v/>
       </c>
@@ -7672,7 +8927,7 @@
           <t>Bevmax cost / case (24)</t>
         </is>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="40">
         <f>D28*D9</f>
         <v/>
       </c>
@@ -7701,7 +8956,7 @@
           <t>Inbound freight to DC</t>
         </is>
       </c>
-      <c r="D34" s="25" t="n">
+      <c r="D34" s="20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7711,7 +8966,7 @@
           <t>Testing / misc</t>
         </is>
       </c>
-      <c r="D35" s="25" t="n">
+      <c r="D35" s="20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7728,7 +8983,7 @@
           <t>OH cost %</t>
         </is>
       </c>
-      <c r="C38" s="34" t="n">
+      <c r="C38" s="21" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -7738,7 +8993,7 @@
           <t>Other COGS %</t>
         </is>
       </c>
-      <c r="C39" s="34" t="n">
+      <c r="C39" s="21" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -7750,46 +9005,46 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="35" t="inlineStr">
+      <c r="A44" s="23" t="inlineStr">
         <is>
           <t>COGS Direct / case</t>
         </is>
       </c>
-      <c r="B44" s="36" t="n"/>
-      <c r="C44" s="36" t="n"/>
-      <c r="D44" s="37">
+      <c r="B44" s="41" t="n"/>
+      <c r="C44" s="41" t="n"/>
+      <c r="D44" s="42">
         <f>D30+D33+D34+D35</f>
         <v/>
       </c>
-      <c r="E44" s="36" t="n"/>
+      <c r="E44" s="41" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="35" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t>COGS Indirect / case</t>
         </is>
       </c>
-      <c r="B45" s="36" t="n"/>
-      <c r="C45" s="36" t="n"/>
-      <c r="D45" s="37">
+      <c r="B45" s="41" t="n"/>
+      <c r="C45" s="41" t="n"/>
+      <c r="D45" s="42">
         <f>(C38+C39)*D44</f>
         <v/>
       </c>
-      <c r="E45" s="36" t="n"/>
+      <c r="E45" s="41" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="35" t="inlineStr">
+      <c r="A46" s="23" t="inlineStr">
         <is>
           <t>COGS Total / case</t>
         </is>
       </c>
-      <c r="B46" s="36" t="n"/>
-      <c r="C46" s="36" t="n"/>
-      <c r="D46" s="37">
+      <c r="B46" s="41" t="n"/>
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="42">
         <f>D44+D45</f>
         <v/>
       </c>
-      <c r="E46" s="36" t="n"/>
+      <c r="E46" s="41" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">

</xml_diff>